<commit_message>
New SSM report template for DX
</commit_message>
<xml_diff>
--- a/Rapportering/Arsstatistik/ReportTemplates/RTG Mall årsredovisning DosReg 2025.xlsx
+++ b/Rapportering/Arsstatistik/ReportTemplates/RTG Mall årsredovisning DosReg 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\rvbrtg\Rapportering\Arsstatistik\ReportTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonsod\Desktop\Till Dosreg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44D2C12E-E957-4F0A-B0F6-9EF5509CA361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{90BD35F5-EAB4-4C55-9CA5-EDEEBA021F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RTG" sheetId="2" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="51">
   <si>
     <t>Kvinnor (16 år och äldre)</t>
   </si>
@@ -180,15 +183,6 @@
     <t>RTG03</t>
   </si>
   <si>
-    <t>Övre buk (exklusive njurar)</t>
-  </si>
-  <si>
-    <t>RTG04</t>
-  </si>
-  <si>
-    <t>Nedre Buk (inklusive njurar, exklusive bäcken/höft)</t>
-  </si>
-  <si>
     <t>RTG05</t>
   </si>
   <si>
@@ -259,6 +253,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Buk</t>
   </si>
 </sst>
 </file>
@@ -341,10 +338,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -352,14 +351,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -640,10 +644,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="45.5703125" customWidth="1"/>
     <col min="5" max="6" width="14.28515625" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -668,42 +674,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="2" customFormat="1" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="7"/>
+      <c r="E1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="12" t="s">
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="8" t="s">
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="12" t="s">
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="3" t="s">
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="T1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="6"/>
-      <c r="X1" s="3" t="s">
+      <c r="V1" s="4"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Y1" s="3" t="s">
@@ -711,19 +717,19 @@
       </c>
     </row>
     <row r="2" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="12" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -741,7 +747,7 @@
       <c r="J2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="8" t="s">
         <v>11</v>
       </c>
       <c r="L2" s="3" t="s">
@@ -762,11 +768,11 @@
       <c r="Q2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="8" t="s">
         <v>11</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>9</v>
@@ -777,11 +783,11 @@
       <c r="V2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="W2" s="6" t="s">
+      <c r="W2" s="8" t="s">
         <v>11</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="Y2" s="3" t="s">
         <v>9</v>
@@ -806,12 +812,12 @@
       <c r="C3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="W3" s="7"/>
+      <c r="K3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -823,12 +829,12 @@
       <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="W4" s="7"/>
+      <c r="K4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -840,16 +846,16 @@
       <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="R5" s="7"/>
-      <c r="W5" s="7"/>
+      <c r="D5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>20</v>
@@ -857,16 +863,16 @@
       <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="W6" s="7"/>
+      <c r="D6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="W6" s="9"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>20</v>
@@ -874,16 +880,16 @@
       <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="7"/>
-      <c r="R7" s="7"/>
-      <c r="W7" s="7"/>
+      <c r="D7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="W7" s="9"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>20</v>
@@ -891,16 +897,16 @@
       <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="W8" s="7"/>
+      <c r="D8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="W8" s="9"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>20</v>
@@ -908,266 +914,254 @@
       <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="7"/>
-      <c r="R9" s="7"/>
-      <c r="W9" s="7"/>
+      <c r="D9" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="P9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="R9" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="U9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="V9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="W9" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB9" s="17" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="K10" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="R10" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="T10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="U10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="V10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="W10" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB10" s="11" t="s">
-        <v>52</v>
-      </c>
+      <c r="D10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="15"/>
+      <c r="K10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="W10" s="9"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K11" s="7"/>
-      <c r="R11" s="7"/>
-      <c r="W11" s="7"/>
+      <c r="D11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="K11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="W11" s="9"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K12" s="7"/>
-      <c r="R12" s="7"/>
-      <c r="W12" s="7"/>
+      <c r="D12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="O12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="P12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="R12" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="U12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="V12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="W12" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB12" s="17" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="T13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="U13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="V13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="W13" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB13" s="11" t="s">
-        <v>52</v>
-      </c>
+      <c r="D13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" s="9"/>
+      <c r="R13" s="9"/>
+      <c r="W13" s="9"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="K14" s="7"/>
-      <c r="R14" s="7"/>
-      <c r="W14" s="7"/>
+        <v>42</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="W14" s="9"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="W15" s="7"/>
+      <c r="H15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="O15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="P15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="R15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="U15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="V15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="W15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB15" s="17" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="P16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="R16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="T16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="U16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="V16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="W16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AA16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB16" s="11" t="s">
-        <v>52</v>
-      </c>
+      <c r="D16" s="1"/>
     </row>
     <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" s="1"/>
@@ -1183,9 +1177,6 @@
     </row>
     <row r="21" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D22" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>